<commit_message>
Enhance Chrome and Edge driver configurations to accept insecure certificates for QA environments
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata/login.xlsx
+++ b/src/main/resources/testdata/login.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Automation Projects\Projects\CareIR-automation\src\main\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BCAA086-3C69-45B0-A99B-9A4AC6D896E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8685F0E7-BC13-4C9D-9483-089A7E13423E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1884" yWindow="1884" windowWidth="17280" windowHeight="8832" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="3">
   <si>
     <t>username</t>
   </si>
@@ -33,28 +33,17 @@
     <t>password</t>
   </si>
   <si>
-    <t>akshay</t>
-  </si>
-  <si>
-    <t>akugale27@</t>
+    <t>vendor</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -77,16 +66,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -366,9 +352,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -376,17 +362,17 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>3</v>
+      <c r="B2" t="s">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{12F436E3-C13B-4FF7-8A4B-5CC0EC9B9681}"/>
+    <hyperlink ref="B2" r:id="rId1" display="akugale27@" xr:uid="{12F436E3-C13B-4FF7-8A4B-5CC0EC9B9681}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>